<commit_message>
feat: add demonic pile tutor mechanics
</commit_message>
<xml_diff>
--- a/game_data.xlsx
+++ b/game_data.xlsx
@@ -5912,7 +5912,7 @@
         </is>
       </c>
       <c r="E79" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F79" s="4" t="inlineStr">
         <is>
@@ -5953,8 +5953,14 @@
       <c r="N79" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="O79" s="3" t="inlineStr"/>
-      <c r="P79" s="4" t="n"/>
+      <c r="O79" s="3" t="inlineStr">
+        <is>
+          <t>牌堆检索</t>
+        </is>
+      </c>
+      <c r="P79" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q79" s="3" t="inlineStr"/>
       <c r="R79" s="4" t="n"/>
     </row>
@@ -8888,7 +8894,7 @@
         </is>
       </c>
       <c r="E123" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F123" s="4" t="inlineStr">
         <is>
@@ -8917,7 +8923,7 @@
       </c>
       <c r="K123" s="3" t="inlineStr">
         <is>
-          <t>抽牌</t>
+          <t>牌堆检索</t>
         </is>
       </c>
       <c r="L123" s="4" t="n">

</xml_diff>

<commit_message>
feat: recover cards from the exhaust pile
</commit_message>
<xml_diff>
--- a/game_data.xlsx
+++ b/game_data.xlsx
@@ -5402,12 +5402,12 @@
       </c>
       <c r="H71" s="4" t="inlineStr">
         <is>
-          <t>蓝</t>
+          <t>金</t>
         </is>
       </c>
       <c r="I71" s="4" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="J71" s="4" t="inlineStr">
@@ -5423,8 +5423,14 @@
       <c r="L71" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="M71" s="3" t="inlineStr"/>
-      <c r="N71" s="4" t="n"/>
+      <c r="M71" s="3" t="inlineStr">
+        <is>
+          <t>牌堆检索</t>
+        </is>
+      </c>
+      <c r="N71" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="O71" s="3" t="inlineStr"/>
       <c r="P71" s="4" t="n"/>
       <c r="Q71" s="3" t="inlineStr"/>

</xml_diff>

<commit_message>
feat: add exhaust-driven demonic defense
</commit_message>
<xml_diff>
--- a/game_data.xlsx
+++ b/game_data.xlsx
@@ -6056,11 +6056,11 @@
         </is>
       </c>
       <c r="E81" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F81" s="4" t="inlineStr">
         <is>
-          <t>技能</t>
+          <t>功法</t>
         </is>
       </c>
       <c r="G81" s="4" t="inlineStr">
@@ -6070,12 +6070,12 @@
       </c>
       <c r="H81" s="4" t="inlineStr">
         <is>
-          <t>白</t>
+          <t>蓝</t>
         </is>
       </c>
       <c r="I81" s="4" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="J81" s="4" t="inlineStr">
@@ -6101,12 +6101,10 @@
       </c>
       <c r="O81" s="3" t="inlineStr">
         <is>
-          <t>灵气</t>
-        </is>
-      </c>
-      <c r="P81" s="4" t="n">
-        <v>1</v>
-      </c>
+          <t>configured_demonic_engine_effect</t>
+        </is>
+      </c>
+      <c r="P81" s="4" t="n"/>
       <c r="Q81" s="3" t="inlineStr"/>
       <c r="R81" s="4" t="n"/>
     </row>
@@ -6735,8 +6733,14 @@
         </is>
       </c>
       <c r="L91" s="4" t="n"/>
-      <c r="M91" s="3" t="inlineStr"/>
-      <c r="N91" s="4" t="n"/>
+      <c r="M91" s="3" t="inlineStr">
+        <is>
+          <t>灵气</t>
+        </is>
+      </c>
+      <c r="N91" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="O91" s="3" t="inlineStr"/>
       <c r="P91" s="4" t="n"/>
       <c r="Q91" s="3" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: sync curse game data
</commit_message>
<xml_diff>
--- a/game_data.xlsx
+++ b/game_data.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R173"/>
+  <dimension ref="A1:R175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -11775,12 +11775,12 @@
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>common_cards/status/eclipse_scar.tres</t>
+          <t>common_cards/status/blood_debt_curse.tres</t>
         </is>
       </c>
       <c r="B165" s="3" t="inlineStr">
         <is>
-          <t>eclipse_scar</t>
+          <t>blood_debt_curse</t>
         </is>
       </c>
       <c r="C165" s="3" t="inlineStr">
@@ -11790,7 +11790,7 @@
       </c>
       <c r="D165" s="4" t="inlineStr">
         <is>
-          <t>蚀痕</t>
+          <t>血债</t>
         </is>
       </c>
       <c r="E165" s="4" t="n">
@@ -11821,8 +11821,14 @@
           <t>无</t>
         </is>
       </c>
-      <c r="K165" s="3" t="inlineStr"/>
-      <c r="L165" s="4" t="n"/>
+      <c r="K165" s="3" t="inlineStr">
+        <is>
+          <t>自损</t>
+        </is>
+      </c>
+      <c r="L165" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="M165" s="3" t="inlineStr"/>
       <c r="N165" s="4" t="n"/>
       <c r="O165" s="3" t="inlineStr"/>
@@ -11833,12 +11839,12 @@
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>common_cards/status/heart_demon.tres</t>
+          <t>common_cards/status/eclipse_scar.tres</t>
         </is>
       </c>
       <c r="B166" s="3" t="inlineStr">
         <is>
-          <t>heart_demon</t>
+          <t>eclipse_scar</t>
         </is>
       </c>
       <c r="C166" s="3" t="inlineStr">
@@ -11848,7 +11854,7 @@
       </c>
       <c r="D166" s="4" t="inlineStr">
         <is>
-          <t>心魔</t>
+          <t>蚀痕</t>
         </is>
       </c>
       <c r="E166" s="4" t="n">
@@ -11891,12 +11897,12 @@
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>common_cards/status/underworld_writ.tres</t>
+          <t>common_cards/status/heart_demon.tres</t>
         </is>
       </c>
       <c r="B167" s="3" t="inlineStr">
         <is>
-          <t>underworld_writ</t>
+          <t>heart_demon</t>
         </is>
       </c>
       <c r="C167" s="3" t="inlineStr">
@@ -11906,7 +11912,7 @@
       </c>
       <c r="D167" s="4" t="inlineStr">
         <is>
-          <t>判牒</t>
+          <t>心魔</t>
         </is>
       </c>
       <c r="E167" s="4" t="n">
@@ -11949,12 +11955,12 @@
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>common_cards/strike.tres</t>
+          <t>common_cards/status/karmic_fire_curse.tres</t>
         </is>
       </c>
       <c r="B168" s="3" t="inlineStr">
         <is>
-          <t>strike</t>
+          <t>karmic_fire_curse</t>
         </is>
       </c>
       <c r="C168" s="3" t="inlineStr">
@@ -11964,7 +11970,7 @@
       </c>
       <c r="D168" s="4" t="inlineStr">
         <is>
-          <t>打击</t>
+          <t>业火</t>
         </is>
       </c>
       <c r="E168" s="4" t="n">
@@ -11972,12 +11978,12 @@
       </c>
       <c r="F168" s="4" t="inlineStr">
         <is>
-          <t>攻击</t>
+          <t>技能</t>
         </is>
       </c>
       <c r="G168" s="4" t="inlineStr">
         <is>
-          <t>单体</t>
+          <t>自身</t>
         </is>
       </c>
       <c r="H168" s="4" t="inlineStr">
@@ -11987,7 +11993,7 @@
       </c>
       <c r="I168" s="4" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="J168" s="4" t="inlineStr">
@@ -11997,11 +12003,11 @@
       </c>
       <c r="K168" s="3" t="inlineStr">
         <is>
-          <t>伤害</t>
+          <t>自损</t>
         </is>
       </c>
       <c r="L168" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M168" s="3" t="inlineStr"/>
       <c r="N168" s="4" t="n"/>
@@ -12013,12 +12019,12 @@
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>common_cards/toxin.tres</t>
+          <t>common_cards/status/underworld_writ.tres</t>
         </is>
       </c>
       <c r="B169" s="3" t="inlineStr">
         <is>
-          <t>toxin</t>
+          <t>underworld_writ</t>
         </is>
       </c>
       <c r="C169" s="3" t="inlineStr">
@@ -12028,11 +12034,11 @@
       </c>
       <c r="D169" s="4" t="inlineStr">
         <is>
-          <t>浊气</t>
+          <t>判牒</t>
         </is>
       </c>
       <c r="E169" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F169" s="4" t="inlineStr">
         <is>
@@ -12051,7 +12057,7 @@
       </c>
       <c r="I169" s="4" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="J169" s="4" t="inlineStr">
@@ -12071,22 +12077,22 @@
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>fusion_cards/attack_guard_unity.tres</t>
+          <t>common_cards/strike.tres</t>
         </is>
       </c>
       <c r="B170" s="3" t="inlineStr">
         <is>
-          <t>attack_guard_unity</t>
+          <t>strike</t>
         </is>
       </c>
       <c r="C170" s="3" t="inlineStr">
         <is>
-          <t>融合</t>
+          <t>通用</t>
         </is>
       </c>
       <c r="D170" s="4" t="inlineStr">
         <is>
-          <t>攻守合一</t>
+          <t>打击</t>
         </is>
       </c>
       <c r="E170" s="4" t="n">
@@ -12104,7 +12110,7 @@
       </c>
       <c r="H170" s="4" t="inlineStr">
         <is>
-          <t>蓝</t>
+          <t>白</t>
         </is>
       </c>
       <c r="I170" s="4" t="inlineStr">
@@ -12125,14 +12131,8 @@
       <c r="L170" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="M170" s="3" t="inlineStr">
-        <is>
-          <t>护体</t>
-        </is>
-      </c>
-      <c r="N170" s="4" t="n">
-        <v>5</v>
-      </c>
+      <c r="M170" s="3" t="inlineStr"/>
+      <c r="N170" s="4" t="n"/>
       <c r="O170" s="3" t="inlineStr"/>
       <c r="P170" s="4" t="n"/>
       <c r="Q170" s="3" t="inlineStr"/>
@@ -12141,22 +12141,22 @@
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>fusion_cards/blood_beast_rend.tres</t>
+          <t>common_cards/toxin.tres</t>
         </is>
       </c>
       <c r="B171" s="3" t="inlineStr">
         <is>
-          <t>blood_beast_rend</t>
+          <t>toxin</t>
         </is>
       </c>
       <c r="C171" s="3" t="inlineStr">
         <is>
-          <t>融合</t>
+          <t>通用</t>
         </is>
       </c>
       <c r="D171" s="4" t="inlineStr">
         <is>
-          <t>血兽撕咬</t>
+          <t>浊气</t>
         </is>
       </c>
       <c r="E171" s="4" t="n">
@@ -12164,45 +12164,33 @@
       </c>
       <c r="F171" s="4" t="inlineStr">
         <is>
-          <t>攻击</t>
+          <t>技能</t>
         </is>
       </c>
       <c r="G171" s="4" t="inlineStr">
         <is>
-          <t>单体</t>
+          <t>自身</t>
         </is>
       </c>
       <c r="H171" s="4" t="inlineStr">
         <is>
-          <t>蓝</t>
+          <t>白</t>
         </is>
       </c>
       <c r="I171" s="4" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="J171" s="4" t="inlineStr">
         <is>
-          <t>火</t>
-        </is>
-      </c>
-      <c r="K171" s="3" t="inlineStr">
-        <is>
-          <t>伤害</t>
-        </is>
-      </c>
-      <c r="L171" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="M171" s="3" t="inlineStr">
-        <is>
-          <t>自损</t>
-        </is>
-      </c>
-      <c r="N171" s="4" t="n">
-        <v>2</v>
-      </c>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="K171" s="3" t="inlineStr"/>
+      <c r="L171" s="4" t="n"/>
+      <c r="M171" s="3" t="inlineStr"/>
+      <c r="N171" s="4" t="n"/>
       <c r="O171" s="3" t="inlineStr"/>
       <c r="P171" s="4" t="n"/>
       <c r="Q171" s="3" t="inlineStr"/>
@@ -12211,12 +12199,12 @@
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>fusion_cards/demon_rain_swordfire.tres</t>
+          <t>fusion_cards/attack_guard_unity.tres</t>
         </is>
       </c>
       <c r="B172" s="3" t="inlineStr">
         <is>
-          <t>demon_rain_swordfire</t>
+          <t>attack_guard_unity</t>
         </is>
       </c>
       <c r="C172" s="3" t="inlineStr">
@@ -12226,11 +12214,11 @@
       </c>
       <c r="D172" s="4" t="inlineStr">
         <is>
-          <t>魔雨剑火</t>
+          <t>攻守合一</t>
         </is>
       </c>
       <c r="E172" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F172" s="4" t="inlineStr">
         <is>
@@ -12239,12 +12227,12 @@
       </c>
       <c r="G172" s="4" t="inlineStr">
         <is>
-          <t>全体敌</t>
+          <t>单体</t>
         </is>
       </c>
       <c r="H172" s="4" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>蓝</t>
         </is>
       </c>
       <c r="I172" s="4" t="inlineStr">
@@ -12254,7 +12242,7 @@
       </c>
       <c r="J172" s="4" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>无</t>
         </is>
       </c>
       <c r="K172" s="3" t="inlineStr">
@@ -12263,15 +12251,15 @@
         </is>
       </c>
       <c r="L172" s="4" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="M172" s="3" t="inlineStr">
         <is>
-          <t>自损</t>
+          <t>护体</t>
         </is>
       </c>
       <c r="N172" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O172" s="3" t="inlineStr"/>
       <c r="P172" s="4" t="n"/>
@@ -12281,12 +12269,12 @@
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
         <is>
-          <t>fusion_cards/sword_shield_chime.tres</t>
+          <t>fusion_cards/blood_beast_rend.tres</t>
         </is>
       </c>
       <c r="B173" s="3" t="inlineStr">
         <is>
-          <t>sword_shield_chime</t>
+          <t>blood_beast_rend</t>
         </is>
       </c>
       <c r="C173" s="3" t="inlineStr">
@@ -12296,7 +12284,7 @@
       </c>
       <c r="D173" s="4" t="inlineStr">
         <is>
-          <t>剑盾合鸣</t>
+          <t>血兽撕咬</t>
         </is>
       </c>
       <c r="E173" s="4" t="n">
@@ -12324,7 +12312,7 @@
       </c>
       <c r="J173" s="4" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>火</t>
         </is>
       </c>
       <c r="K173" s="3" t="inlineStr">
@@ -12333,42 +12321,182 @@
         </is>
       </c>
       <c r="L173" s="4" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="M173" s="3" t="inlineStr">
         <is>
-          <t>护体</t>
+          <t>自损</t>
         </is>
       </c>
       <c r="N173" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="O173" s="3" t="inlineStr">
-        <is>
-          <t>抽牌</t>
-        </is>
-      </c>
-      <c r="P173" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="O173" s="3" t="inlineStr"/>
+      <c r="P173" s="4" t="n"/>
       <c r="Q173" s="3" t="inlineStr"/>
       <c r="R173" s="4" t="n"/>
     </row>
+    <row r="174">
+      <c r="A174" s="2" t="inlineStr">
+        <is>
+          <t>fusion_cards/demon_rain_swordfire.tres</t>
+        </is>
+      </c>
+      <c r="B174" s="3" t="inlineStr">
+        <is>
+          <t>demon_rain_swordfire</t>
+        </is>
+      </c>
+      <c r="C174" s="3" t="inlineStr">
+        <is>
+          <t>融合</t>
+        </is>
+      </c>
+      <c r="D174" s="4" t="inlineStr">
+        <is>
+          <t>魔雨剑火</t>
+        </is>
+      </c>
+      <c r="E174" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F174" s="4" t="inlineStr">
+        <is>
+          <t>攻击</t>
+        </is>
+      </c>
+      <c r="G174" s="4" t="inlineStr">
+        <is>
+          <t>全体敌</t>
+        </is>
+      </c>
+      <c r="H174" s="4" t="inlineStr">
+        <is>
+          <t>金</t>
+        </is>
+      </c>
+      <c r="I174" s="4" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J174" s="4" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="K174" s="3" t="inlineStr">
+        <is>
+          <t>伤害</t>
+        </is>
+      </c>
+      <c r="L174" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="M174" s="3" t="inlineStr">
+        <is>
+          <t>自损</t>
+        </is>
+      </c>
+      <c r="N174" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O174" s="3" t="inlineStr"/>
+      <c r="P174" s="4" t="n"/>
+      <c r="Q174" s="3" t="inlineStr"/>
+      <c r="R174" s="4" t="n"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="inlineStr">
+        <is>
+          <t>fusion_cards/sword_shield_chime.tres</t>
+        </is>
+      </c>
+      <c r="B175" s="3" t="inlineStr">
+        <is>
+          <t>sword_shield_chime</t>
+        </is>
+      </c>
+      <c r="C175" s="3" t="inlineStr">
+        <is>
+          <t>融合</t>
+        </is>
+      </c>
+      <c r="D175" s="4" t="inlineStr">
+        <is>
+          <t>剑盾合鸣</t>
+        </is>
+      </c>
+      <c r="E175" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F175" s="4" t="inlineStr">
+        <is>
+          <t>攻击</t>
+        </is>
+      </c>
+      <c r="G175" s="4" t="inlineStr">
+        <is>
+          <t>单体</t>
+        </is>
+      </c>
+      <c r="H175" s="4" t="inlineStr">
+        <is>
+          <t>蓝</t>
+        </is>
+      </c>
+      <c r="I175" s="4" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J175" s="4" t="inlineStr">
+        <is>
+          <t>金</t>
+        </is>
+      </c>
+      <c r="K175" s="3" t="inlineStr">
+        <is>
+          <t>伤害</t>
+        </is>
+      </c>
+      <c r="L175" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="M175" s="3" t="inlineStr">
+        <is>
+          <t>护体</t>
+        </is>
+      </c>
+      <c r="N175" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="O175" s="3" t="inlineStr">
+        <is>
+          <t>抽牌</t>
+        </is>
+      </c>
+      <c r="P175" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q175" s="3" t="inlineStr"/>
+      <c r="R175" s="4" t="n"/>
+    </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation sqref="F2:F173" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F175" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"攻击,技能,功法"</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G173" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G2:G175" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"自身,单体,全体敌,所有"</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H173" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H175" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"白,蓝,金,暗金"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I173" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I175" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"是,否"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J173" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J175" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"无,金,木,水,火,土"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat: add combat card count scaling
</commit_message>
<xml_diff>
--- a/game_data.xlsx
+++ b/game_data.xlsx
@@ -8025,12 +8025,10 @@
       </c>
       <c r="K110" s="3" t="inlineStr">
         <is>
-          <t>伤害</t>
-        </is>
-      </c>
-      <c r="L110" s="4" t="n">
-        <v>4</v>
-      </c>
+          <t>计数增幅</t>
+        </is>
+      </c>
+      <c r="L110" s="4" t="n"/>
       <c r="M110" s="3" t="inlineStr">
         <is>
           <t>状态(soul_mark)</t>
@@ -8801,11 +8799,11 @@
       </c>
       <c r="K121" s="3" t="inlineStr">
         <is>
-          <t>半血爆伤</t>
+          <t>计数增幅</t>
         </is>
       </c>
       <c r="L121" s="4" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="M121" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: complete common card construction pool
</commit_message>
<xml_diff>
--- a/game_data.xlsx
+++ b/game_data.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R175"/>
+  <dimension ref="A1:R183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -11569,12 +11569,12 @@
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>common_cards/defend.tres</t>
+          <t>common_cards/ash_heart_guard.tres</t>
         </is>
       </c>
       <c r="B162" s="3" t="inlineStr">
         <is>
-          <t>defend</t>
+          <t>ash_heart_guard</t>
         </is>
       </c>
       <c r="C162" s="3" t="inlineStr">
@@ -11584,7 +11584,7 @@
       </c>
       <c r="D162" s="4" t="inlineStr">
         <is>
-          <t>防御</t>
+          <t>灰烬护心</t>
         </is>
       </c>
       <c r="E162" s="4" t="n">
@@ -11602,7 +11602,7 @@
       </c>
       <c r="H162" s="4" t="inlineStr">
         <is>
-          <t>白</t>
+          <t>蓝</t>
         </is>
       </c>
       <c r="I162" s="4" t="inlineStr">
@@ -11617,11 +11617,11 @@
       </c>
       <c r="K162" s="3" t="inlineStr">
         <is>
-          <t>护体</t>
+          <t>计数增幅</t>
         </is>
       </c>
       <c r="L162" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M162" s="3" t="inlineStr"/>
       <c r="N162" s="4" t="n"/>
@@ -11633,12 +11633,12 @@
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>common_cards/ink_flow_slash.tres</t>
+          <t>common_cards/circulating_breath.tres</t>
         </is>
       </c>
       <c r="B163" s="3" t="inlineStr">
         <is>
-          <t>ink_flow_slash</t>
+          <t>circulating_breath</t>
         </is>
       </c>
       <c r="C163" s="3" t="inlineStr">
@@ -11648,7 +11648,7 @@
       </c>
       <c r="D163" s="4" t="inlineStr">
         <is>
-          <t>墨流斩</t>
+          <t>周天吐纳</t>
         </is>
       </c>
       <c r="E163" s="4" t="n">
@@ -11656,12 +11656,12 @@
       </c>
       <c r="F163" s="4" t="inlineStr">
         <is>
-          <t>攻击</t>
+          <t>技能</t>
         </is>
       </c>
       <c r="G163" s="4" t="inlineStr">
         <is>
-          <t>单体</t>
+          <t>自身</t>
         </is>
       </c>
       <c r="H163" s="4" t="inlineStr">
@@ -11681,7 +11681,7 @@
       </c>
       <c r="K163" s="3" t="inlineStr">
         <is>
-          <t>伤害</t>
+          <t>护体</t>
         </is>
       </c>
       <c r="L163" s="4" t="n">
@@ -11703,12 +11703,12 @@
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>common_cards/muscle_resonance_strike.tres</t>
+          <t>common_cards/defend.tres</t>
         </is>
       </c>
       <c r="B164" s="3" t="inlineStr">
         <is>
-          <t>muscle_resonance_strike</t>
+          <t>defend</t>
         </is>
       </c>
       <c r="C164" s="3" t="inlineStr">
@@ -11718,7 +11718,7 @@
       </c>
       <c r="D164" s="4" t="inlineStr">
         <is>
-          <t>劲气共鸣</t>
+          <t>防御</t>
         </is>
       </c>
       <c r="E164" s="4" t="n">
@@ -11726,12 +11726,12 @@
       </c>
       <c r="F164" s="4" t="inlineStr">
         <is>
-          <t>攻击</t>
+          <t>技能</t>
         </is>
       </c>
       <c r="G164" s="4" t="inlineStr">
         <is>
-          <t>单体</t>
+          <t>自身</t>
         </is>
       </c>
       <c r="H164" s="4" t="inlineStr">
@@ -11751,20 +11751,14 @@
       </c>
       <c r="K164" s="3" t="inlineStr">
         <is>
-          <t>伤害</t>
+          <t>护体</t>
         </is>
       </c>
       <c r="L164" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="M164" s="3" t="inlineStr">
-        <is>
-          <t>伤害</t>
-        </is>
-      </c>
-      <c r="N164" s="4" t="n">
-        <v>4</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="M164" s="3" t="inlineStr"/>
+      <c r="N164" s="4" t="n"/>
       <c r="O164" s="3" t="inlineStr"/>
       <c r="P164" s="4" t="n"/>
       <c r="Q164" s="3" t="inlineStr"/>
@@ -11773,12 +11767,12 @@
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>common_cards/status/blood_debt_curse.tres</t>
+          <t>common_cards/discard_aegis.tres</t>
         </is>
       </c>
       <c r="B165" s="3" t="inlineStr">
         <is>
-          <t>blood_debt_curse</t>
+          <t>discard_aegis</t>
         </is>
       </c>
       <c r="C165" s="3" t="inlineStr">
@@ -11788,11 +11782,11 @@
       </c>
       <c r="D165" s="4" t="inlineStr">
         <is>
-          <t>血债</t>
+          <t>弃念成罡</t>
         </is>
       </c>
       <c r="E165" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F165" s="4" t="inlineStr">
         <is>
@@ -11806,7 +11800,7 @@
       </c>
       <c r="H165" s="4" t="inlineStr">
         <is>
-          <t>白</t>
+          <t>金</t>
         </is>
       </c>
       <c r="I165" s="4" t="inlineStr">
@@ -11821,11 +11815,11 @@
       </c>
       <c r="K165" s="3" t="inlineStr">
         <is>
-          <t>自损</t>
+          <t>计数增幅</t>
         </is>
       </c>
       <c r="L165" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M165" s="3" t="inlineStr"/>
       <c r="N165" s="4" t="n"/>
@@ -11837,12 +11831,12 @@
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>common_cards/status/eclipse_scar.tres</t>
+          <t>common_cards/embers_return.tres</t>
         </is>
       </c>
       <c r="B166" s="3" t="inlineStr">
         <is>
-          <t>eclipse_scar</t>
+          <t>embers_return</t>
         </is>
       </c>
       <c r="C166" s="3" t="inlineStr">
@@ -11852,11 +11846,11 @@
       </c>
       <c r="D166" s="4" t="inlineStr">
         <is>
-          <t>蚀痕</t>
+          <t>烬归灵台</t>
         </is>
       </c>
       <c r="E166" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F166" s="4" t="inlineStr">
         <is>
@@ -11870,12 +11864,12 @@
       </c>
       <c r="H166" s="4" t="inlineStr">
         <is>
-          <t>白</t>
+          <t>蓝</t>
         </is>
       </c>
       <c r="I166" s="4" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="J166" s="4" t="inlineStr">
@@ -11883,10 +11877,22 @@
           <t>无</t>
         </is>
       </c>
-      <c r="K166" s="3" t="inlineStr"/>
-      <c r="L166" s="4" t="n"/>
-      <c r="M166" s="3" t="inlineStr"/>
-      <c r="N166" s="4" t="n"/>
+      <c r="K166" s="3" t="inlineStr">
+        <is>
+          <t>护体</t>
+        </is>
+      </c>
+      <c r="L166" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M166" s="3" t="inlineStr">
+        <is>
+          <t>抽牌</t>
+        </is>
+      </c>
+      <c r="N166" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="O166" s="3" t="inlineStr"/>
       <c r="P166" s="4" t="n"/>
       <c r="Q166" s="3" t="inlineStr"/>
@@ -11895,12 +11901,12 @@
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>common_cards/status/heart_demon.tres</t>
+          <t>common_cards/flowing_cloud_guard.tres</t>
         </is>
       </c>
       <c r="B167" s="3" t="inlineStr">
         <is>
-          <t>heart_demon</t>
+          <t>flowing_cloud_guard</t>
         </is>
       </c>
       <c r="C167" s="3" t="inlineStr">
@@ -11910,11 +11916,11 @@
       </c>
       <c r="D167" s="4" t="inlineStr">
         <is>
-          <t>心魔</t>
+          <t>流云护身</t>
         </is>
       </c>
       <c r="E167" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F167" s="4" t="inlineStr">
         <is>
@@ -11928,7 +11934,7 @@
       </c>
       <c r="H167" s="4" t="inlineStr">
         <is>
-          <t>白</t>
+          <t>蓝</t>
         </is>
       </c>
       <c r="I167" s="4" t="inlineStr">
@@ -11941,7 +11947,11 @@
           <t>无</t>
         </is>
       </c>
-      <c r="K167" s="3" t="inlineStr"/>
+      <c r="K167" s="3" t="inlineStr">
+        <is>
+          <t>计数增幅</t>
+        </is>
+      </c>
       <c r="L167" s="4" t="n"/>
       <c r="M167" s="3" t="inlineStr"/>
       <c r="N167" s="4" t="n"/>
@@ -11953,12 +11963,12 @@
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>common_cards/status/karmic_fire_curse.tres</t>
+          <t>common_cards/ink_flow_slash.tres</t>
         </is>
       </c>
       <c r="B168" s="3" t="inlineStr">
         <is>
-          <t>karmic_fire_curse</t>
+          <t>ink_flow_slash</t>
         </is>
       </c>
       <c r="C168" s="3" t="inlineStr">
@@ -11968,7 +11978,7 @@
       </c>
       <c r="D168" s="4" t="inlineStr">
         <is>
-          <t>业火</t>
+          <t>墨流斩</t>
         </is>
       </c>
       <c r="E168" s="4" t="n">
@@ -11976,12 +11986,12 @@
       </c>
       <c r="F168" s="4" t="inlineStr">
         <is>
-          <t>技能</t>
+          <t>攻击</t>
         </is>
       </c>
       <c r="G168" s="4" t="inlineStr">
         <is>
-          <t>自身</t>
+          <t>单体</t>
         </is>
       </c>
       <c r="H168" s="4" t="inlineStr">
@@ -11991,7 +12001,7 @@
       </c>
       <c r="I168" s="4" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="J168" s="4" t="inlineStr">
@@ -12001,14 +12011,20 @@
       </c>
       <c r="K168" s="3" t="inlineStr">
         <is>
-          <t>自损</t>
+          <t>伤害</t>
         </is>
       </c>
       <c r="L168" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="M168" s="3" t="inlineStr"/>
-      <c r="N168" s="4" t="n"/>
+        <v>5</v>
+      </c>
+      <c r="M168" s="3" t="inlineStr">
+        <is>
+          <t>抽牌</t>
+        </is>
+      </c>
+      <c r="N168" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="O168" s="3" t="inlineStr"/>
       <c r="P168" s="4" t="n"/>
       <c r="Q168" s="3" t="inlineStr"/>
@@ -12017,12 +12033,12 @@
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>common_cards/status/underworld_writ.tres</t>
+          <t>common_cards/momentum_pursuit.tres</t>
         </is>
       </c>
       <c r="B169" s="3" t="inlineStr">
         <is>
-          <t>underworld_writ</t>
+          <t>momentum_pursuit</t>
         </is>
       </c>
       <c r="C169" s="3" t="inlineStr">
@@ -12032,25 +12048,25 @@
       </c>
       <c r="D169" s="4" t="inlineStr">
         <is>
-          <t>判牒</t>
+          <t>乘势追击</t>
         </is>
       </c>
       <c r="E169" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F169" s="4" t="inlineStr">
         <is>
-          <t>技能</t>
+          <t>攻击</t>
         </is>
       </c>
       <c r="G169" s="4" t="inlineStr">
         <is>
-          <t>自身</t>
+          <t>单体</t>
         </is>
       </c>
       <c r="H169" s="4" t="inlineStr">
         <is>
-          <t>白</t>
+          <t>蓝</t>
         </is>
       </c>
       <c r="I169" s="4" t="inlineStr">
@@ -12063,8 +12079,14 @@
           <t>无</t>
         </is>
       </c>
-      <c r="K169" s="3" t="inlineStr"/>
-      <c r="L169" s="4" t="n"/>
+      <c r="K169" s="3" t="inlineStr">
+        <is>
+          <t>计数增幅</t>
+        </is>
+      </c>
+      <c r="L169" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="M169" s="3" t="inlineStr"/>
       <c r="N169" s="4" t="n"/>
       <c r="O169" s="3" t="inlineStr"/>
@@ -12075,12 +12097,12 @@
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>common_cards/strike.tres</t>
+          <t>common_cards/muscle_resonance_strike.tres</t>
         </is>
       </c>
       <c r="B170" s="3" t="inlineStr">
         <is>
-          <t>strike</t>
+          <t>muscle_resonance_strike</t>
         </is>
       </c>
       <c r="C170" s="3" t="inlineStr">
@@ -12090,7 +12112,7 @@
       </c>
       <c r="D170" s="4" t="inlineStr">
         <is>
-          <t>打击</t>
+          <t>劲气共鸣</t>
         </is>
       </c>
       <c r="E170" s="4" t="n">
@@ -12127,10 +12149,16 @@
         </is>
       </c>
       <c r="L170" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="M170" s="3" t="inlineStr"/>
-      <c r="N170" s="4" t="n"/>
+        <v>4</v>
+      </c>
+      <c r="M170" s="3" t="inlineStr">
+        <is>
+          <t>伤害</t>
+        </is>
+      </c>
+      <c r="N170" s="4" t="n">
+        <v>4</v>
+      </c>
       <c r="O170" s="3" t="inlineStr"/>
       <c r="P170" s="4" t="n"/>
       <c r="Q170" s="3" t="inlineStr"/>
@@ -12139,12 +12167,12 @@
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>common_cards/toxin.tres</t>
+          <t>common_cards/returning_light.tres</t>
         </is>
       </c>
       <c r="B171" s="3" t="inlineStr">
         <is>
-          <t>toxin</t>
+          <t>returning_light</t>
         </is>
       </c>
       <c r="C171" s="3" t="inlineStr">
@@ -12154,7 +12182,7 @@
       </c>
       <c r="D171" s="4" t="inlineStr">
         <is>
-          <t>浊气</t>
+          <t>回光返照</t>
         </is>
       </c>
       <c r="E171" s="4" t="n">
@@ -12172,7 +12200,7 @@
       </c>
       <c r="H171" s="4" t="inlineStr">
         <is>
-          <t>白</t>
+          <t>蓝</t>
         </is>
       </c>
       <c r="I171" s="4" t="inlineStr">
@@ -12185,8 +12213,14 @@
           <t>无</t>
         </is>
       </c>
-      <c r="K171" s="3" t="inlineStr"/>
-      <c r="L171" s="4" t="n"/>
+      <c r="K171" s="3" t="inlineStr">
+        <is>
+          <t>治疗</t>
+        </is>
+      </c>
+      <c r="L171" s="4" t="n">
+        <v>5</v>
+      </c>
       <c r="M171" s="3" t="inlineStr"/>
       <c r="N171" s="4" t="n"/>
       <c r="O171" s="3" t="inlineStr"/>
@@ -12197,26 +12231,26 @@
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>fusion_cards/attack_guard_unity.tres</t>
+          <t>common_cards/spirit_stone_needle.tres</t>
         </is>
       </c>
       <c r="B172" s="3" t="inlineStr">
         <is>
-          <t>attack_guard_unity</t>
+          <t>spirit_stone_needle</t>
         </is>
       </c>
       <c r="C172" s="3" t="inlineStr">
         <is>
-          <t>融合</t>
+          <t>通用</t>
         </is>
       </c>
       <c r="D172" s="4" t="inlineStr">
         <is>
-          <t>攻守合一</t>
+          <t>灵石飞针</t>
         </is>
       </c>
       <c r="E172" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F172" s="4" t="inlineStr">
         <is>
@@ -12230,12 +12264,12 @@
       </c>
       <c r="H172" s="4" t="inlineStr">
         <is>
-          <t>蓝</t>
+          <t>白</t>
         </is>
       </c>
       <c r="I172" s="4" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="J172" s="4" t="inlineStr">
@@ -12249,16 +12283,10 @@
         </is>
       </c>
       <c r="L172" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="M172" s="3" t="inlineStr">
-        <is>
-          <t>护体</t>
-        </is>
-      </c>
-      <c r="N172" s="4" t="n">
-        <v>5</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="M172" s="3" t="inlineStr"/>
+      <c r="N172" s="4" t="n"/>
       <c r="O172" s="3" t="inlineStr"/>
       <c r="P172" s="4" t="n"/>
       <c r="Q172" s="3" t="inlineStr"/>
@@ -12267,40 +12295,40 @@
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
         <is>
-          <t>fusion_cards/blood_beast_rend.tres</t>
+          <t>common_cards/status/blood_debt_curse.tres</t>
         </is>
       </c>
       <c r="B173" s="3" t="inlineStr">
         <is>
-          <t>blood_beast_rend</t>
+          <t>blood_debt_curse</t>
         </is>
       </c>
       <c r="C173" s="3" t="inlineStr">
         <is>
-          <t>融合</t>
+          <t>通用</t>
         </is>
       </c>
       <c r="D173" s="4" t="inlineStr">
         <is>
-          <t>血兽撕咬</t>
+          <t>血债</t>
         </is>
       </c>
       <c r="E173" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F173" s="4" t="inlineStr">
         <is>
-          <t>攻击</t>
+          <t>技能</t>
         </is>
       </c>
       <c r="G173" s="4" t="inlineStr">
         <is>
-          <t>单体</t>
+          <t>自身</t>
         </is>
       </c>
       <c r="H173" s="4" t="inlineStr">
         <is>
-          <t>蓝</t>
+          <t>白</t>
         </is>
       </c>
       <c r="I173" s="4" t="inlineStr">
@@ -12310,25 +12338,19 @@
       </c>
       <c r="J173" s="4" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>无</t>
         </is>
       </c>
       <c r="K173" s="3" t="inlineStr">
         <is>
-          <t>伤害</t>
+          <t>自损</t>
         </is>
       </c>
       <c r="L173" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="M173" s="3" t="inlineStr">
-        <is>
-          <t>自损</t>
-        </is>
-      </c>
-      <c r="N173" s="4" t="n">
         <v>2</v>
       </c>
+      <c r="M173" s="3" t="inlineStr"/>
+      <c r="N173" s="4" t="n"/>
       <c r="O173" s="3" t="inlineStr"/>
       <c r="P173" s="4" t="n"/>
       <c r="Q173" s="3" t="inlineStr"/>
@@ -12337,40 +12359,40 @@
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>fusion_cards/demon_rain_swordfire.tres</t>
+          <t>common_cards/status/eclipse_scar.tres</t>
         </is>
       </c>
       <c r="B174" s="3" t="inlineStr">
         <is>
-          <t>demon_rain_swordfire</t>
+          <t>eclipse_scar</t>
         </is>
       </c>
       <c r="C174" s="3" t="inlineStr">
         <is>
-          <t>融合</t>
+          <t>通用</t>
         </is>
       </c>
       <c r="D174" s="4" t="inlineStr">
         <is>
-          <t>魔雨剑火</t>
+          <t>蚀痕</t>
         </is>
       </c>
       <c r="E174" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F174" s="4" t="inlineStr">
         <is>
-          <t>攻击</t>
+          <t>技能</t>
         </is>
       </c>
       <c r="G174" s="4" t="inlineStr">
         <is>
-          <t>全体敌</t>
+          <t>自身</t>
         </is>
       </c>
       <c r="H174" s="4" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>白</t>
         </is>
       </c>
       <c r="I174" s="4" t="inlineStr">
@@ -12380,25 +12402,13 @@
       </c>
       <c r="J174" s="4" t="inlineStr">
         <is>
-          <t>火</t>
-        </is>
-      </c>
-      <c r="K174" s="3" t="inlineStr">
-        <is>
-          <t>伤害</t>
-        </is>
-      </c>
-      <c r="L174" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="M174" s="3" t="inlineStr">
-        <is>
-          <t>自损</t>
-        </is>
-      </c>
-      <c r="N174" s="4" t="n">
-        <v>1</v>
-      </c>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="K174" s="3" t="inlineStr"/>
+      <c r="L174" s="4" t="n"/>
+      <c r="M174" s="3" t="inlineStr"/>
+      <c r="N174" s="4" t="n"/>
       <c r="O174" s="3" t="inlineStr"/>
       <c r="P174" s="4" t="n"/>
       <c r="Q174" s="3" t="inlineStr"/>
@@ -12407,40 +12417,40 @@
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>fusion_cards/sword_shield_chime.tres</t>
+          <t>common_cards/status/heart_demon.tres</t>
         </is>
       </c>
       <c r="B175" s="3" t="inlineStr">
         <is>
-          <t>sword_shield_chime</t>
+          <t>heart_demon</t>
         </is>
       </c>
       <c r="C175" s="3" t="inlineStr">
         <is>
-          <t>融合</t>
+          <t>通用</t>
         </is>
       </c>
       <c r="D175" s="4" t="inlineStr">
         <is>
-          <t>剑盾合鸣</t>
+          <t>心魔</t>
         </is>
       </c>
       <c r="E175" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F175" s="4" t="inlineStr">
         <is>
-          <t>攻击</t>
+          <t>技能</t>
         </is>
       </c>
       <c r="G175" s="4" t="inlineStr">
         <is>
-          <t>单体</t>
+          <t>自身</t>
         </is>
       </c>
       <c r="H175" s="4" t="inlineStr">
         <is>
-          <t>蓝</t>
+          <t>白</t>
         </is>
       </c>
       <c r="I175" s="4" t="inlineStr">
@@ -12450,51 +12460,563 @@
       </c>
       <c r="J175" s="4" t="inlineStr">
         <is>
-          <t>金</t>
-        </is>
-      </c>
-      <c r="K175" s="3" t="inlineStr">
-        <is>
-          <t>伤害</t>
-        </is>
-      </c>
-      <c r="L175" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="M175" s="3" t="inlineStr">
-        <is>
-          <t>护体</t>
-        </is>
-      </c>
-      <c r="N175" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="O175" s="3" t="inlineStr">
-        <is>
-          <t>抽牌</t>
-        </is>
-      </c>
-      <c r="P175" s="4" t="n">
-        <v>1</v>
-      </c>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="K175" s="3" t="inlineStr"/>
+      <c r="L175" s="4" t="n"/>
+      <c r="M175" s="3" t="inlineStr"/>
+      <c r="N175" s="4" t="n"/>
+      <c r="O175" s="3" t="inlineStr"/>
+      <c r="P175" s="4" t="n"/>
       <c r="Q175" s="3" t="inlineStr"/>
       <c r="R175" s="4" t="n"/>
     </row>
+    <row r="176">
+      <c r="A176" s="2" t="inlineStr">
+        <is>
+          <t>common_cards/status/karmic_fire_curse.tres</t>
+        </is>
+      </c>
+      <c r="B176" s="3" t="inlineStr">
+        <is>
+          <t>karmic_fire_curse</t>
+        </is>
+      </c>
+      <c r="C176" s="3" t="inlineStr">
+        <is>
+          <t>通用</t>
+        </is>
+      </c>
+      <c r="D176" s="4" t="inlineStr">
+        <is>
+          <t>业火</t>
+        </is>
+      </c>
+      <c r="E176" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F176" s="4" t="inlineStr">
+        <is>
+          <t>技能</t>
+        </is>
+      </c>
+      <c r="G176" s="4" t="inlineStr">
+        <is>
+          <t>自身</t>
+        </is>
+      </c>
+      <c r="H176" s="4" t="inlineStr">
+        <is>
+          <t>白</t>
+        </is>
+      </c>
+      <c r="I176" s="4" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="J176" s="4" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="K176" s="3" t="inlineStr">
+        <is>
+          <t>自损</t>
+        </is>
+      </c>
+      <c r="L176" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M176" s="3" t="inlineStr"/>
+      <c r="N176" s="4" t="n"/>
+      <c r="O176" s="3" t="inlineStr"/>
+      <c r="P176" s="4" t="n"/>
+      <c r="Q176" s="3" t="inlineStr"/>
+      <c r="R176" s="4" t="n"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="inlineStr">
+        <is>
+          <t>common_cards/status/underworld_writ.tres</t>
+        </is>
+      </c>
+      <c r="B177" s="3" t="inlineStr">
+        <is>
+          <t>underworld_writ</t>
+        </is>
+      </c>
+      <c r="C177" s="3" t="inlineStr">
+        <is>
+          <t>通用</t>
+        </is>
+      </c>
+      <c r="D177" s="4" t="inlineStr">
+        <is>
+          <t>判牒</t>
+        </is>
+      </c>
+      <c r="E177" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F177" s="4" t="inlineStr">
+        <is>
+          <t>技能</t>
+        </is>
+      </c>
+      <c r="G177" s="4" t="inlineStr">
+        <is>
+          <t>自身</t>
+        </is>
+      </c>
+      <c r="H177" s="4" t="inlineStr">
+        <is>
+          <t>白</t>
+        </is>
+      </c>
+      <c r="I177" s="4" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J177" s="4" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="K177" s="3" t="inlineStr"/>
+      <c r="L177" s="4" t="n"/>
+      <c r="M177" s="3" t="inlineStr"/>
+      <c r="N177" s="4" t="n"/>
+      <c r="O177" s="3" t="inlineStr"/>
+      <c r="P177" s="4" t="n"/>
+      <c r="Q177" s="3" t="inlineStr"/>
+      <c r="R177" s="4" t="n"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="inlineStr">
+        <is>
+          <t>common_cards/strike.tres</t>
+        </is>
+      </c>
+      <c r="B178" s="3" t="inlineStr">
+        <is>
+          <t>strike</t>
+        </is>
+      </c>
+      <c r="C178" s="3" t="inlineStr">
+        <is>
+          <t>通用</t>
+        </is>
+      </c>
+      <c r="D178" s="4" t="inlineStr">
+        <is>
+          <t>打击</t>
+        </is>
+      </c>
+      <c r="E178" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F178" s="4" t="inlineStr">
+        <is>
+          <t>攻击</t>
+        </is>
+      </c>
+      <c r="G178" s="4" t="inlineStr">
+        <is>
+          <t>单体</t>
+        </is>
+      </c>
+      <c r="H178" s="4" t="inlineStr">
+        <is>
+          <t>白</t>
+        </is>
+      </c>
+      <c r="I178" s="4" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J178" s="4" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="K178" s="3" t="inlineStr">
+        <is>
+          <t>伤害</t>
+        </is>
+      </c>
+      <c r="L178" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="M178" s="3" t="inlineStr"/>
+      <c r="N178" s="4" t="n"/>
+      <c r="O178" s="3" t="inlineStr"/>
+      <c r="P178" s="4" t="n"/>
+      <c r="Q178" s="3" t="inlineStr"/>
+      <c r="R178" s="4" t="n"/>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="inlineStr">
+        <is>
+          <t>common_cards/toxin.tres</t>
+        </is>
+      </c>
+      <c r="B179" s="3" t="inlineStr">
+        <is>
+          <t>toxin</t>
+        </is>
+      </c>
+      <c r="C179" s="3" t="inlineStr">
+        <is>
+          <t>通用</t>
+        </is>
+      </c>
+      <c r="D179" s="4" t="inlineStr">
+        <is>
+          <t>浊气</t>
+        </is>
+      </c>
+      <c r="E179" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F179" s="4" t="inlineStr">
+        <is>
+          <t>技能</t>
+        </is>
+      </c>
+      <c r="G179" s="4" t="inlineStr">
+        <is>
+          <t>自身</t>
+        </is>
+      </c>
+      <c r="H179" s="4" t="inlineStr">
+        <is>
+          <t>白</t>
+        </is>
+      </c>
+      <c r="I179" s="4" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="J179" s="4" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="K179" s="3" t="inlineStr"/>
+      <c r="L179" s="4" t="n"/>
+      <c r="M179" s="3" t="inlineStr"/>
+      <c r="N179" s="4" t="n"/>
+      <c r="O179" s="3" t="inlineStr"/>
+      <c r="P179" s="4" t="n"/>
+      <c r="Q179" s="3" t="inlineStr"/>
+      <c r="R179" s="4" t="n"/>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>fusion_cards/attack_guard_unity.tres</t>
+        </is>
+      </c>
+      <c r="B180" s="3" t="inlineStr">
+        <is>
+          <t>attack_guard_unity</t>
+        </is>
+      </c>
+      <c r="C180" s="3" t="inlineStr">
+        <is>
+          <t>融合</t>
+        </is>
+      </c>
+      <c r="D180" s="4" t="inlineStr">
+        <is>
+          <t>攻守合一</t>
+        </is>
+      </c>
+      <c r="E180" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F180" s="4" t="inlineStr">
+        <is>
+          <t>攻击</t>
+        </is>
+      </c>
+      <c r="G180" s="4" t="inlineStr">
+        <is>
+          <t>单体</t>
+        </is>
+      </c>
+      <c r="H180" s="4" t="inlineStr">
+        <is>
+          <t>蓝</t>
+        </is>
+      </c>
+      <c r="I180" s="4" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J180" s="4" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="K180" s="3" t="inlineStr">
+        <is>
+          <t>伤害</t>
+        </is>
+      </c>
+      <c r="L180" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="M180" s="3" t="inlineStr">
+        <is>
+          <t>护体</t>
+        </is>
+      </c>
+      <c r="N180" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="O180" s="3" t="inlineStr"/>
+      <c r="P180" s="4" t="n"/>
+      <c r="Q180" s="3" t="inlineStr"/>
+      <c r="R180" s="4" t="n"/>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
+        <is>
+          <t>fusion_cards/blood_beast_rend.tres</t>
+        </is>
+      </c>
+      <c r="B181" s="3" t="inlineStr">
+        <is>
+          <t>blood_beast_rend</t>
+        </is>
+      </c>
+      <c r="C181" s="3" t="inlineStr">
+        <is>
+          <t>融合</t>
+        </is>
+      </c>
+      <c r="D181" s="4" t="inlineStr">
+        <is>
+          <t>血兽撕咬</t>
+        </is>
+      </c>
+      <c r="E181" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F181" s="4" t="inlineStr">
+        <is>
+          <t>攻击</t>
+        </is>
+      </c>
+      <c r="G181" s="4" t="inlineStr">
+        <is>
+          <t>单体</t>
+        </is>
+      </c>
+      <c r="H181" s="4" t="inlineStr">
+        <is>
+          <t>蓝</t>
+        </is>
+      </c>
+      <c r="I181" s="4" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J181" s="4" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="K181" s="3" t="inlineStr">
+        <is>
+          <t>伤害</t>
+        </is>
+      </c>
+      <c r="L181" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="M181" s="3" t="inlineStr">
+        <is>
+          <t>自损</t>
+        </is>
+      </c>
+      <c r="N181" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="O181" s="3" t="inlineStr"/>
+      <c r="P181" s="4" t="n"/>
+      <c r="Q181" s="3" t="inlineStr"/>
+      <c r="R181" s="4" t="n"/>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>fusion_cards/demon_rain_swordfire.tres</t>
+        </is>
+      </c>
+      <c r="B182" s="3" t="inlineStr">
+        <is>
+          <t>demon_rain_swordfire</t>
+        </is>
+      </c>
+      <c r="C182" s="3" t="inlineStr">
+        <is>
+          <t>融合</t>
+        </is>
+      </c>
+      <c r="D182" s="4" t="inlineStr">
+        <is>
+          <t>魔雨剑火</t>
+        </is>
+      </c>
+      <c r="E182" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F182" s="4" t="inlineStr">
+        <is>
+          <t>攻击</t>
+        </is>
+      </c>
+      <c r="G182" s="4" t="inlineStr">
+        <is>
+          <t>全体敌</t>
+        </is>
+      </c>
+      <c r="H182" s="4" t="inlineStr">
+        <is>
+          <t>金</t>
+        </is>
+      </c>
+      <c r="I182" s="4" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J182" s="4" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="K182" s="3" t="inlineStr">
+        <is>
+          <t>伤害</t>
+        </is>
+      </c>
+      <c r="L182" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="M182" s="3" t="inlineStr">
+        <is>
+          <t>自损</t>
+        </is>
+      </c>
+      <c r="N182" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O182" s="3" t="inlineStr"/>
+      <c r="P182" s="4" t="n"/>
+      <c r="Q182" s="3" t="inlineStr"/>
+      <c r="R182" s="4" t="n"/>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr">
+        <is>
+          <t>fusion_cards/sword_shield_chime.tres</t>
+        </is>
+      </c>
+      <c r="B183" s="3" t="inlineStr">
+        <is>
+          <t>sword_shield_chime</t>
+        </is>
+      </c>
+      <c r="C183" s="3" t="inlineStr">
+        <is>
+          <t>融合</t>
+        </is>
+      </c>
+      <c r="D183" s="4" t="inlineStr">
+        <is>
+          <t>剑盾合鸣</t>
+        </is>
+      </c>
+      <c r="E183" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F183" s="4" t="inlineStr">
+        <is>
+          <t>攻击</t>
+        </is>
+      </c>
+      <c r="G183" s="4" t="inlineStr">
+        <is>
+          <t>单体</t>
+        </is>
+      </c>
+      <c r="H183" s="4" t="inlineStr">
+        <is>
+          <t>蓝</t>
+        </is>
+      </c>
+      <c r="I183" s="4" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J183" s="4" t="inlineStr">
+        <is>
+          <t>金</t>
+        </is>
+      </c>
+      <c r="K183" s="3" t="inlineStr">
+        <is>
+          <t>伤害</t>
+        </is>
+      </c>
+      <c r="L183" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="M183" s="3" t="inlineStr">
+        <is>
+          <t>护体</t>
+        </is>
+      </c>
+      <c r="N183" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="O183" s="3" t="inlineStr">
+        <is>
+          <t>抽牌</t>
+        </is>
+      </c>
+      <c r="P183" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q183" s="3" t="inlineStr"/>
+      <c r="R183" s="4" t="n"/>
+    </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation sqref="F2:F175" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F183" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"攻击,技能,功法"</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G175" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G2:G183" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"自身,单体,全体敌,所有"</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H175" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H183" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"白,蓝,金,暗金"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I175" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I183" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"是,否"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J175" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J183" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"无,金,木,水,火,土"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>